<commit_message>
Sync final PNAS analysis code and data
</commit_message>
<xml_diff>
--- a/Code/TCS_scripts_EN/TCS_scripts_EN_1/ED_Fig_3_droplet_morphometry.xlsx
+++ b/Code/TCS_scripts_EN/TCS_scripts_EN_1/ED_Fig_3_droplet_morphometry.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary_stats" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Droplet_measurements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scale_beads" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bias_curve" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Volume_distribution" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary_stats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Droplet_measurements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Scale_beads" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bias_curve" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Volume_distribution" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,13 +22,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -39,7 +42,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,12 +50,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,7 +434,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ED Fig. 3 droplet morphometry</t>
         </is>
@@ -506,22 +518,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>quantity</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -942,47 +954,47 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>droplet_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cx_px</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>cy_px</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>r_px</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>diameter_um</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>volume_fL</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>n_beads_inside</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>weight_1_over_V</t>
         </is>
@@ -13000,32 +13012,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>bead_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>cx_px</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>cy_px</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>r_px</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>diameter_um</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -20570,12 +20582,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>volume_fL</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>concentration_bias_pct</t>
         </is>
@@ -23796,12 +23808,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>volume_fL</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>distribution_density_norm</t>
         </is>
@@ -23868,7 +23880,7 @@
         <v>16.08383030464838</v>
       </c>
       <c r="B9" t="n">
-        <v>0.2265783126266643</v>
+        <v>0.2265783126266644</v>
       </c>
     </row>
     <row r="10">
@@ -23892,7 +23904,7 @@
         <v>16.57198132405566</v>
       </c>
       <c r="B12" t="n">
-        <v>0.2516938553459767</v>
+        <v>0.2516938553459768</v>
       </c>
     </row>
     <row r="13">
@@ -23908,7 +23920,7 @@
         <v>16.90561873986437</v>
       </c>
       <c r="B14" t="n">
-        <v>0.2691583461725575</v>
+        <v>0.2691583461725576</v>
       </c>
     </row>
     <row r="15">
@@ -23924,7 +23936,7 @@
         <v>17.24597315124836</v>
       </c>
       <c r="B16" t="n">
-        <v>0.2871358054028039</v>
+        <v>0.2871358054028038</v>
       </c>
     </row>
     <row r="17">
@@ -23940,7 +23952,7 @@
         <v>17.59317978893245</v>
       </c>
       <c r="B18" t="n">
-        <v>0.3055744464521502</v>
+        <v>0.3055744464521503</v>
       </c>
     </row>
     <row r="19">
@@ -23956,7 +23968,7 @@
         <v>17.94737660619033</v>
       </c>
       <c r="B20" t="n">
-        <v>0.3244262769878425</v>
+        <v>0.3244262769878424</v>
       </c>
     </row>
     <row r="21">
@@ -23964,7 +23976,7 @@
         <v>18.1271402004708</v>
       </c>
       <c r="B21" t="n">
-        <v>0.3339934156784272</v>
+        <v>0.3339934156784273</v>
       </c>
     </row>
     <row r="22">
@@ -23972,7 +23984,7 @@
         <v>18.30870433365662</v>
       </c>
       <c r="B22" t="n">
-        <v>0.3436480410867512</v>
+        <v>0.3436480410867511</v>
       </c>
     </row>
     <row r="23">
@@ -23988,7 +24000,7 @@
         <v>18.6773065352425</v>
       </c>
       <c r="B24" t="n">
-        <v>0.3632018799397564</v>
+        <v>0.3632018799397565</v>
       </c>
     </row>
     <row r="25">
@@ -24004,7 +24016,7 @@
         <v>19.05332966517688</v>
       </c>
       <c r="B26" t="n">
-        <v>0.3830556801748125</v>
+        <v>0.3830556801748126</v>
       </c>
     </row>
     <row r="27">
@@ -24028,7 +24040,7 @@
         <v>19.63160624003423</v>
       </c>
       <c r="B29" t="n">
-        <v>0.4133426716161382</v>
+        <v>0.4133426716161383</v>
       </c>
     </row>
     <row r="30">
@@ -24036,7 +24048,7 @@
         <v>19.82823932890529</v>
       </c>
       <c r="B30" t="n">
-        <v>0.4235632100573289</v>
+        <v>0.423563210057329</v>
       </c>
     </row>
     <row r="31">
@@ -24052,7 +24064,7 @@
         <v>20.2274337523343</v>
       </c>
       <c r="B32" t="n">
-        <v>0.444179936254076</v>
+        <v>0.4441799362540761</v>
       </c>
     </row>
     <row r="33">
@@ -24076,7 +24088,7 @@
         <v>20.84134488041561</v>
       </c>
       <c r="B35" t="n">
-        <v>0.4755226667384986</v>
+        <v>0.4755226667384987</v>
       </c>
     </row>
     <row r="36">
@@ -24084,7 +24096,7 @@
         <v>21.05009489149245</v>
       </c>
       <c r="B36" t="n">
-        <v>0.4860769357450767</v>
+        <v>0.4860769357450769</v>
       </c>
     </row>
     <row r="37">
@@ -24116,7 +24128,7 @@
         <v>21.90621412316829</v>
       </c>
       <c r="B40" t="n">
-        <v>0.528799577943033</v>
+        <v>0.5287995779430328</v>
       </c>
     </row>
     <row r="41">
@@ -24124,7 +24136,7 @@
         <v>22.12563002301072</v>
       </c>
       <c r="B41" t="n">
-        <v>0.53960073101394</v>
+        <v>0.5396007310139401</v>
       </c>
     </row>
     <row r="42">
@@ -24132,7 +24144,7 @@
         <v>22.34724362515046</v>
       </c>
       <c r="B42" t="n">
-        <v>0.5504471546390844</v>
+        <v>0.5504471546390846</v>
       </c>
     </row>
     <row r="43">
@@ -24140,7 +24152,7 @@
         <v>22.57107694210067</v>
       </c>
       <c r="B43" t="n">
-        <v>0.5613369596993969</v>
+        <v>0.5613369596993971</v>
       </c>
     </row>
     <row r="44">
@@ -24148,7 +24160,7 @@
         <v>22.79715220685516</v>
       </c>
       <c r="B44" t="n">
-        <v>0.5722679352045542</v>
+        <v>0.5722679352045541</v>
       </c>
     </row>
     <row r="45">
@@ -24156,7 +24168,7 @@
         <v>23.0254918750967</v>
       </c>
       <c r="B45" t="n">
-        <v>0.583237502275484</v>
+        <v>0.5832375022754839</v>
       </c>
     </row>
     <row r="46">
@@ -24172,7 +24184,7 @@
         <v>23.48905537162202</v>
       </c>
       <c r="B47" t="n">
-        <v>0.6052800002751112</v>
+        <v>0.605280000275111</v>
       </c>
     </row>
     <row r="48">
@@ -24180,7 +24192,7 @@
         <v>23.72432524490252</v>
       </c>
       <c r="B48" t="n">
-        <v>0.6163455623066698</v>
+        <v>0.6163455623066699</v>
       </c>
     </row>
     <row r="49">
@@ -24188,7 +24200,7 @@
         <v>23.96195161623701</v>
       </c>
       <c r="B49" t="n">
-        <v>0.6274349102113307</v>
+        <v>0.6274349102113308</v>
       </c>
     </row>
     <row r="50">
@@ -24204,7 +24216,7 @@
         <v>24.44436850161992</v>
       </c>
       <c r="B51" t="n">
-        <v>0.6496644237953665</v>
+        <v>0.6496644237953666</v>
       </c>
     </row>
     <row r="52">
@@ -24212,7 +24224,7 @@
         <v>24.68920693334101</v>
       </c>
       <c r="B52" t="n">
-        <v>0.6607928818449762</v>
+        <v>0.6607928818449763</v>
       </c>
     </row>
     <row r="53">
@@ -24220,7 +24232,7 @@
         <v>24.93649770322104</v>
       </c>
       <c r="B53" t="n">
-        <v>0.6719216820387007</v>
+        <v>0.671921682038701</v>
       </c>
     </row>
     <row r="54">
@@ -24236,7 +24248,7 @@
         <v>25.43853475541984</v>
       </c>
       <c r="B55" t="n">
-        <v>0.6941503229226795</v>
+        <v>0.6941503229226798</v>
       </c>
     </row>
     <row r="56">
@@ -24244,7 +24256,7 @@
         <v>25.69333090425006</v>
       </c>
       <c r="B56" t="n">
-        <v>0.7052336696709585</v>
+        <v>0.7052336696709587</v>
       </c>
     </row>
     <row r="57">
@@ -24260,7 +24272,7 @@
         <v>26.21060499228978</v>
       </c>
       <c r="B58" t="n">
-        <v>0.7272927786528212</v>
+        <v>0.7272927786528213</v>
       </c>
     </row>
     <row r="59">
@@ -24268,7 +24280,7 @@
         <v>26.47313431148033</v>
       </c>
       <c r="B59" t="n">
-        <v>0.7382485974208731</v>
+        <v>0.7382485974208732</v>
       </c>
     </row>
     <row r="60">
@@ -24276,7 +24288,7 @@
         <v>26.73829316339074</v>
       </c>
       <c r="B60" t="n">
-        <v>0.7491410827071425</v>
+        <v>0.7491410827071426</v>
       </c>
     </row>
     <row r="61">
@@ -24300,7 +24312,7 @@
         <v>27.54981161500906</v>
       </c>
       <c r="B63" t="n">
-        <v>0.781323900280282</v>
+        <v>0.7813239002802819</v>
       </c>
     </row>
     <row r="64">
@@ -24316,7 +24328,7 @@
         <v>28.10446152521055</v>
       </c>
       <c r="B65" t="n">
-        <v>0.8022452569178603</v>
+        <v>0.8022452569178605</v>
       </c>
     </row>
     <row r="66">
@@ -24324,7 +24336,7 @@
         <v>28.38595999320093</v>
       </c>
       <c r="B66" t="n">
-        <v>0.8125075793448796</v>
+        <v>0.8125075793448795</v>
       </c>
     </row>
     <row r="67">
@@ -24340,7 +24352,7 @@
         <v>28.95744376162839</v>
       </c>
       <c r="B68" t="n">
-        <v>0.832569570403923</v>
+        <v>0.8325695704039233</v>
       </c>
     </row>
     <row r="69">
@@ -24348,7 +24360,7 @@
         <v>29.24748582660458</v>
       </c>
       <c r="B69" t="n">
-        <v>0.8423424932374155</v>
+        <v>0.8423424932374154</v>
       </c>
     </row>
     <row r="70">
@@ -24364,7 +24376,7 @@
         <v>29.83631436794054</v>
       </c>
       <c r="B71" t="n">
-        <v>0.8613051443533017</v>
+        <v>0.8613051443533019</v>
       </c>
     </row>
     <row r="72">
@@ -24372,7 +24384,7 @@
         <v>30.13515933166705</v>
       </c>
       <c r="B72" t="n">
-        <v>0.8704682434265357</v>
+        <v>0.8704682434265359</v>
       </c>
     </row>
     <row r="73">
@@ -24388,7 +24400,7 @@
         <v>30.74185906706962</v>
       </c>
       <c r="B74" t="n">
-        <v>0.8880926501901848</v>
+        <v>0.8880926501901849</v>
       </c>
     </row>
     <row r="75">
@@ -24396,7 +24408,7 @@
         <v>31.04977410122867</v>
       </c>
       <c r="B75" t="n">
-        <v>0.8965285786397931</v>
+        <v>0.8965285786397933</v>
       </c>
     </row>
     <row r="76">
@@ -24404,7 +24416,7 @@
         <v>31.36077325818112</v>
       </c>
       <c r="B76" t="n">
-        <v>0.9046972998229339</v>
+        <v>0.9046972998229341</v>
       </c>
     </row>
     <row r="77">
@@ -24412,7 +24424,7 @@
         <v>31.67488742895976</v>
       </c>
       <c r="B77" t="n">
-        <v>0.9125870553507223</v>
+        <v>0.9125870553507224</v>
       </c>
     </row>
     <row r="78">
@@ -24420,7 +24432,7 @@
         <v>31.99214781400651</v>
       </c>
       <c r="B78" t="n">
-        <v>0.9201865618005449</v>
+        <v>0.920186561800545</v>
       </c>
     </row>
     <row r="79">
@@ -24428,7 +24440,7 @@
         <v>32.31258592627158</v>
       </c>
       <c r="B79" t="n">
-        <v>0.9274850637659161</v>
+        <v>0.9274850637659164</v>
       </c>
     </row>
     <row r="80">
@@ -24436,7 +24448,7 @@
         <v>32.63623359434356</v>
       </c>
       <c r="B80" t="n">
-        <v>0.9344723839617026</v>
+        <v>0.934472383961703</v>
       </c>
     </row>
     <row r="81">
@@ -24444,7 +24456,7 @@
         <v>32.96312296561092</v>
       </c>
       <c r="B81" t="n">
-        <v>0.9411389701179318</v>
+        <v>0.9411389701179317</v>
       </c>
     </row>
     <row r="82">
@@ -24452,7 +24464,7 @@
         <v>33.29328650945517</v>
       </c>
       <c r="B82" t="n">
-        <v>0.9474759384323909</v>
+        <v>0.9474759384323911</v>
       </c>
     </row>
     <row r="83">
@@ -24460,7 +24472,7 @@
         <v>33.62675702047599</v>
       </c>
       <c r="B83" t="n">
-        <v>0.9534751133891445</v>
+        <v>0.9534751133891448</v>
       </c>
     </row>
     <row r="84">
@@ -24476,7 +24488,7 @@
         <v>34.30375176811388</v>
       </c>
       <c r="B85" t="n">
-        <v>0.9644311348545859</v>
+        <v>0.9644311348545862</v>
       </c>
     </row>
     <row r="86">
@@ -24484,7 +24496,7 @@
         <v>34.64734324950143</v>
       </c>
       <c r="B86" t="n">
-        <v>0.9693754763725739</v>
+        <v>0.9693754763725736</v>
       </c>
     </row>
     <row r="87">
@@ -24492,7 +24504,7 @@
         <v>34.99437619428575</v>
       </c>
       <c r="B87" t="n">
-        <v>0.9739570667360693</v>
+        <v>0.973957066736069</v>
       </c>
     </row>
     <row r="88">
@@ -24500,7 +24512,7 @@
         <v>35.34488507267626</v>
       </c>
       <c r="B88" t="n">
-        <v>0.9781717329447429</v>
+        <v>0.9781717329447431</v>
       </c>
     </row>
     <row r="89">
@@ -24508,7 +24520,7 @@
         <v>35.69890470014109</v>
       </c>
       <c r="B89" t="n">
-        <v>0.9820161665160397</v>
+        <v>0.98201616651604</v>
       </c>
     </row>
     <row r="90">
@@ -24516,7 +24528,7 @@
         <v>36.05647024086528</v>
       </c>
       <c r="B90" t="n">
-        <v>0.9854879353514486</v>
+        <v>0.985487935351449</v>
       </c>
     </row>
     <row r="91">
@@ -24524,7 +24536,7 @@
         <v>36.41761721124362</v>
       </c>
       <c r="B91" t="n">
-        <v>0.9885854916049107</v>
+        <v>0.988585491604911</v>
       </c>
     </row>
     <row r="92">
@@ -24540,7 +24552,7 @@
         <v>37.15079928879235</v>
       </c>
       <c r="B93" t="n">
-        <v>0.9936562160337712</v>
+        <v>0.9936562160337715</v>
       </c>
     </row>
     <row r="94">
@@ -24548,7 +24560,7 @@
         <v>37.52290722172791</v>
       </c>
       <c r="B94" t="n">
-        <v>0.9956307261054006</v>
+        <v>0.9956307261054007</v>
       </c>
     </row>
     <row r="95">
@@ -24556,7 +24568,7 @@
         <v>37.89874224308161</v>
       </c>
       <c r="B95" t="n">
-        <v>0.9972336964446107</v>
+        <v>0.9972336964446109</v>
       </c>
     </row>
     <row r="96">
@@ -24564,7 +24576,7 @@
         <v>38.27834168392556</v>
       </c>
       <c r="B96" t="n">
-        <v>0.9984679841901106</v>
+        <v>0.9984679841901101</v>
       </c>
     </row>
     <row r="97">
@@ -24572,7 +24584,7 @@
         <v>38.66174324924542</v>
       </c>
       <c r="B97" t="n">
-        <v>0.999337298800385</v>
+        <v>0.9993372988003849</v>
       </c>
     </row>
     <row r="98">
@@ -24604,7 +24616,7 @@
         <v>40.2341381527558</v>
       </c>
       <c r="B101" t="n">
-        <v>0.9992677801370203</v>
+        <v>0.9992677801370204</v>
       </c>
     </row>
     <row r="102">
@@ -24612,7 +24624,7 @@
         <v>40.63712926648892</v>
       </c>
       <c r="B102" t="n">
-        <v>0.9983963057829637</v>
+        <v>0.9983963057829639</v>
       </c>
     </row>
     <row r="103">
@@ -24636,7 +24648,7 @@
         <v>41.87048324383651</v>
       </c>
       <c r="B105" t="n">
-        <v>0.9938625324595322</v>
+        <v>0.9938625324595319</v>
       </c>
     </row>
     <row r="106">
@@ -24652,7 +24664,7 @@
         <v>42.71344580546197</v>
       </c>
       <c r="B107" t="n">
-        <v>0.9893384069741625</v>
+        <v>0.9893384069741629</v>
       </c>
     </row>
     <row r="108">
@@ -24660,7 +24672,7 @@
         <v>43.14127003351352</v>
       </c>
       <c r="B108" t="n">
-        <v>0.9866581930344482</v>
+        <v>0.9866581930344481</v>
       </c>
     </row>
     <row r="109">
@@ -24668,7 +24680,7 @@
         <v>43.57337941268452</v>
       </c>
       <c r="B109" t="n">
-        <v>0.9837147445720875</v>
+        <v>0.9837147445720879</v>
       </c>
     </row>
     <row r="110">
@@ -24676,7 +24688,7 @@
         <v>44.00981686368608</v>
       </c>
       <c r="B110" t="n">
-        <v>0.9805202431452074</v>
+        <v>0.9805202431452077</v>
       </c>
     </row>
     <row r="111">
@@ -24684,7 +24696,7 @@
         <v>44.4506257371296</v>
       </c>
       <c r="B111" t="n">
-        <v>0.9770872379581905</v>
+        <v>0.9770872379581902</v>
       </c>
     </row>
     <row r="112">
@@ -24700,7 +24712,7 @@
         <v>45.34553332916799</v>
       </c>
       <c r="B113" t="n">
-        <v>0.969557450460753</v>
+        <v>0.9695574504607529</v>
       </c>
     </row>
     <row r="114">
@@ -24708,7 +24720,7 @@
         <v>45.79972093745637</v>
       </c>
       <c r="B114" t="n">
-        <v>0.9654871490258625</v>
+        <v>0.9654871490258627</v>
       </c>
     </row>
     <row r="115">
@@ -24716,7 +24728,7 @@
         <v>46.25845775640293</v>
       </c>
       <c r="B115" t="n">
-        <v>0.9612311998302642</v>
+        <v>0.9612311998302643</v>
       </c>
     </row>
     <row r="116">
@@ -24724,7 +24736,7 @@
         <v>46.72178935157846</v>
       </c>
       <c r="B116" t="n">
-        <v>0.9568032176522132</v>
+        <v>0.9568032176522134</v>
       </c>
     </row>
     <row r="117">
@@ -24732,7 +24744,7 @@
         <v>47.18976174494528</v>
       </c>
       <c r="B117" t="n">
-        <v>0.9522168691110108</v>
+        <v>0.9522168691110106</v>
       </c>
     </row>
     <row r="118">
@@ -24740,7 +24752,7 @@
         <v>47.66242141942853</v>
       </c>
       <c r="B118" t="n">
-        <v>0.9474858175603678</v>
+        <v>0.9474858175603679</v>
       </c>
     </row>
     <row r="119">
@@ -24748,7 +24760,7 @@
         <v>48.13981532353325</v>
       </c>
       <c r="B119" t="n">
-        <v>0.942623667835791</v>
+        <v>0.9426236678357911</v>
       </c>
     </row>
     <row r="120">
@@ -24756,7 +24768,7 @@
         <v>48.62199087600767</v>
       </c>
       <c r="B120" t="n">
-        <v>0.9376439110961535</v>
+        <v>0.9376439110961539</v>
       </c>
     </row>
     <row r="121">
@@ -24764,7 +24776,7 @@
         <v>49.10899597055327</v>
       </c>
       <c r="B121" t="n">
-        <v>0.932559870012531</v>
+        <v>0.9325598700125313</v>
       </c>
     </row>
     <row r="122">
@@ -24772,7 +24784,7 @@
         <v>49.600878980582</v>
       </c>
       <c r="B122" t="n">
-        <v>0.9273846445695765</v>
+        <v>0.9273846445695767</v>
       </c>
     </row>
     <row r="123">
@@ -24780,7 +24792,7 @@
         <v>50.09768876402102</v>
       </c>
       <c r="B123" t="n">
-        <v>0.9221310587555835</v>
+        <v>0.9221310587555838</v>
       </c>
     </row>
     <row r="124">
@@ -24788,7 +24800,7 @@
         <v>50.59947466816583</v>
       </c>
       <c r="B124" t="n">
-        <v>0.9168116084268306</v>
+        <v>0.9168116084268308</v>
       </c>
     </row>
     <row r="125">
@@ -24796,7 +24808,7 @@
         <v>51.10628653458176</v>
       </c>
       <c r="B125" t="n">
-        <v>0.9114384106393388</v>
+        <v>0.9114384106393389</v>
       </c>
     </row>
     <row r="126">
@@ -24804,7 +24816,7 @@
         <v>51.61817470405471</v>
       </c>
       <c r="B126" t="n">
-        <v>0.9060231547465094</v>
+        <v>0.9060231547465093</v>
       </c>
     </row>
     <row r="127">
@@ -24812,7 +24824,7 @@
         <v>52.13519002159128</v>
       </c>
       <c r="B127" t="n">
-        <v>0.9005770555638991</v>
+        <v>0.9005770555638994</v>
       </c>
     </row>
     <row r="128">
@@ -24820,7 +24832,7 @@
         <v>52.65738384146933</v>
       </c>
       <c r="B128" t="n">
-        <v>0.8951108089025749</v>
+        <v>0.8951108089025752</v>
       </c>
     </row>
     <row r="129">
@@ -24828,7 +24840,7 @@
         <v>53.18480803233876</v>
       </c>
       <c r="B129" t="n">
-        <v>0.8896345497694649</v>
+        <v>0.8896345497694652</v>
       </c>
     </row>
     <row r="130">
@@ -24836,7 +24848,7 @@
         <v>53.71751498237357</v>
       </c>
       <c r="B130" t="n">
-        <v>0.8841578135271383</v>
+        <v>0.8841578135271381</v>
       </c>
     </row>
     <row r="131">
@@ -24844,7 +24856,7 @@
         <v>54.25555760447556</v>
       </c>
       <c r="B131" t="n">
-        <v>0.8786895002960208</v>
+        <v>0.8786895002960209</v>
       </c>
     </row>
     <row r="132">
@@ -24852,7 +24864,7 @@
         <v>54.79898934152995</v>
       </c>
       <c r="B132" t="n">
-        <v>0.8732378428692832</v>
+        <v>0.8732378428692834</v>
       </c>
     </row>
     <row r="133">
@@ -24860,7 +24872,7 @@
         <v>55.34786417171392</v>
       </c>
       <c r="B133" t="n">
-        <v>0.8678103783944651</v>
+        <v>0.8678103783944654</v>
       </c>
     </row>
     <row r="134">
@@ -24868,7 +24880,7 @@
         <v>55.90223661385807</v>
       </c>
       <c r="B134" t="n">
-        <v>0.8624139240562829</v>
+        <v>0.8624139240562831</v>
       </c>
     </row>
     <row r="135">
@@ -24876,7 +24888,7 @@
         <v>56.46216173286174</v>
       </c>
       <c r="B135" t="n">
-        <v>0.8570545569721881</v>
+        <v>0.8570545569721885</v>
       </c>
     </row>
     <row r="136">
@@ -24884,7 +24896,7 @@
         <v>57.02769514516242</v>
       </c>
       <c r="B136" t="n">
-        <v>0.8517375984861242</v>
+        <v>0.8517375984861237</v>
       </c>
     </row>
     <row r="137">
@@ -24892,7 +24904,7 @@
         <v>57.59889302426021</v>
       </c>
       <c r="B137" t="n">
-        <v>0.8464676030168425</v>
+        <v>0.8464676030168429</v>
       </c>
     </row>
     <row r="138">
@@ -24900,7 +24912,7 @@
         <v>58.17581210629729</v>
       </c>
       <c r="B138" t="n">
-        <v>0.8412483515853546</v>
+        <v>0.8412483515853547</v>
       </c>
     </row>
     <row r="139">
@@ -24908,7 +24920,7 @@
         <v>58.75850969569354</v>
       </c>
       <c r="B139" t="n">
-        <v>0.8360828501116997</v>
+        <v>0.8360828501117</v>
       </c>
     </row>
     <row r="140">
@@ -24924,7 +24936,7 @@
         <v>59.94147248983965</v>
       </c>
       <c r="B141" t="n">
-        <v>0.8259212687718839</v>
+        <v>0.8259212687718841</v>
       </c>
     </row>
     <row r="142">
@@ -24932,7 +24944,7 @@
         <v>60.54185519633062</v>
       </c>
       <c r="B142" t="n">
-        <v>0.8209273774910983</v>
+        <v>0.8209273774910982</v>
       </c>
     </row>
     <row r="143">
@@ -24940,7 +24952,7 @@
         <v>61.14825142533415</v>
       </c>
       <c r="B143" t="n">
-        <v>0.8159916436374445</v>
+        <v>0.8159916436374446</v>
       </c>
     </row>
     <row r="144">
@@ -24948,7 +24960,7 @@
         <v>61.76072140918641</v>
       </c>
       <c r="B144" t="n">
-        <v>0.8111133406027823</v>
+        <v>0.8111133406027822</v>
       </c>
     </row>
     <row r="145">
@@ -24956,7 +24968,7 @@
         <v>62.37932598351961</v>
       </c>
       <c r="B145" t="n">
-        <v>0.80629105689681</v>
+        <v>0.8062910568968098</v>
       </c>
     </row>
     <row r="146">
@@ -24964,7 +24976,7 @@
         <v>63.0041265933047</v>
       </c>
       <c r="B146" t="n">
-        <v>0.8015227271324376</v>
+        <v>0.8015227271324377</v>
       </c>
     </row>
     <row r="147">
@@ -24972,7 +24984,7 @@
         <v>63.63518529895462</v>
       </c>
       <c r="B147" t="n">
-        <v>0.7968056671007899</v>
+        <v>0.79680566710079</v>
       </c>
     </row>
     <row r="148">
@@ -24980,7 +24992,7 @@
         <v>64.27256478248864</v>
       </c>
       <c r="B148" t="n">
-        <v>0.7921366126736061</v>
+        <v>0.7921366126736065</v>
       </c>
     </row>
     <row r="149">
@@ -24988,7 +25000,7 @@
         <v>64.9163283537584</v>
       </c>
       <c r="B149" t="n">
-        <v>0.787511762235247</v>
+        <v>0.7875117622352472</v>
       </c>
     </row>
     <row r="150">
@@ -24996,7 +25008,7 @@
         <v>65.56653995673651</v>
       </c>
       <c r="B150" t="n">
-        <v>0.782926822313697</v>
+        <v>0.7829268223136971</v>
       </c>
     </row>
     <row r="151">
@@ -25004,7 +25016,7 @@
         <v>66.2232641758679</v>
       </c>
       <c r="B151" t="n">
-        <v>0.7783770560499714</v>
+        <v>0.7783770560499715</v>
       </c>
     </row>
     <row r="152">
@@ -25012,7 +25024,7 @@
         <v>66.88656624248486</v>
       </c>
       <c r="B152" t="n">
-        <v>0.7738573341187293</v>
+        <v>0.7738573341187295</v>
       </c>
     </row>
     <row r="153">
@@ -25028,7 +25040,7 @@
         <v>68.23316811688277</v>
       </c>
       <c r="B154" t="n">
-        <v>0.7648858630035105</v>
+        <v>0.7648858630035106</v>
       </c>
     </row>
     <row r="155">
@@ -25036,7 +25048,7 @@
         <v>68.91660168040445</v>
       </c>
       <c r="B155" t="n">
-        <v>0.7604223771111517</v>
+        <v>0.7604223771111515</v>
       </c>
     </row>
     <row r="156">
@@ -25044,7 +25056,7 @@
         <v>69.60688061617893</v>
       </c>
       <c r="B156" t="n">
-        <v>0.7559655743360697</v>
+        <v>0.7559655743360698</v>
       </c>
     </row>
     <row r="157">
@@ -25052,7 +25064,7 @@
         <v>70.30407348847314</v>
       </c>
       <c r="B157" t="n">
-        <v>0.7515091829879297</v>
+        <v>0.7515091829879298</v>
       </c>
     </row>
     <row r="158">
@@ -25060,7 +25072,7 @@
         <v>71.00824954830391</v>
       </c>
       <c r="B158" t="n">
-        <v>0.7470468718763379</v>
+        <v>0.7470468718763378</v>
       </c>
     </row>
     <row r="159">
@@ -25068,7 +25080,7 @@
         <v>71.71947874031656</v>
       </c>
       <c r="B159" t="n">
-        <v>0.7425723061672334</v>
+        <v>0.7425723061672332</v>
       </c>
     </row>
     <row r="160">
@@ -25076,7 +25088,7 @@
         <v>72.43783170973238</v>
       </c>
       <c r="B160" t="n">
-        <v>0.7380792021366235</v>
+        <v>0.7380792021366237</v>
       </c>
     </row>
     <row r="161">
@@ -25092,7 +25104,7 @@
         <v>73.89619510671135</v>
       </c>
       <c r="B162" t="n">
-        <v>0.7290128171318215</v>
+        <v>0.7290128171318216</v>
       </c>
     </row>
     <row r="163">
@@ -25100,7 +25112,7 @@
         <v>74.63635039110268</v>
       </c>
       <c r="B163" t="n">
-        <v>0.7244276931000989</v>
+        <v>0.724427693100099</v>
       </c>
     </row>
     <row r="164">
@@ -25116,7 +25128,7 @@
         <v>76.13897573100301</v>
       </c>
       <c r="B165" t="n">
-        <v>0.7151257826536792</v>
+        <v>0.7151257826536793</v>
       </c>
     </row>
     <row r="166">
@@ -25124,7 +25136,7 @@
         <v>76.90159503980593</v>
       </c>
       <c r="B166" t="n">
-        <v>0.7103987809362706</v>
+        <v>0.7103987809362707</v>
       </c>
     </row>
     <row r="167">
@@ -25132,7 +25144,7 @@
         <v>77.67185285706755</v>
       </c>
       <c r="B167" t="n">
-        <v>0.7056148639419806</v>
+        <v>0.7056148639419807</v>
       </c>
     </row>
     <row r="168">
@@ -25140,7 +25152,7 @@
         <v>78.44982569122506</v>
       </c>
       <c r="B168" t="n">
-        <v>0.7007698634489665</v>
+        <v>0.7007698634489667</v>
       </c>
     </row>
     <row r="169">
@@ -25156,7 +25168,7 @@
         <v>80.02922628325145</v>
       </c>
       <c r="B170" t="n">
-        <v>0.6908821177711703</v>
+        <v>0.6908821177711704</v>
       </c>
     </row>
     <row r="171">
@@ -25172,7 +25184,7 @@
         <v>81.64042434847951</v>
       </c>
       <c r="B172" t="n">
-        <v>0.6807112226744538</v>
+        <v>0.6807112226744539</v>
       </c>
     </row>
     <row r="173">
@@ -25196,7 +25208,7 @@
         <v>84.11824558979387</v>
       </c>
       <c r="B175" t="n">
-        <v>0.6648900926439436</v>
+        <v>0.6648900926439437</v>
       </c>
     </row>
     <row r="176">
@@ -25204,7 +25216,7 @@
         <v>84.96078645265028</v>
       </c>
       <c r="B176" t="n">
-        <v>0.6594620903289191</v>
+        <v>0.659462090328919</v>
       </c>
     </row>
     <row r="177">
@@ -25212,7 +25224,7 @@
         <v>85.8117663301415</v>
       </c>
       <c r="B177" t="n">
-        <v>0.6539568930512258</v>
+        <v>0.6539568930512255</v>
       </c>
     </row>
     <row r="178">
@@ -25228,7 +25240,7 @@
         <v>87.53938208136189</v>
       </c>
       <c r="B179" t="n">
-        <v>0.6427182807681574</v>
+        <v>0.6427182807681576</v>
       </c>
     </row>
     <row r="180">
@@ -25244,7 +25256,7 @@
         <v>89.30177926538001</v>
       </c>
       <c r="B181" t="n">
-        <v>0.6311857325980852</v>
+        <v>0.6311857325980853</v>
       </c>
     </row>
     <row r="182">
@@ -25260,7 +25272,7 @@
         <v>91.09965812359304</v>
       </c>
       <c r="B183" t="n">
-        <v>0.6193778902879097</v>
+        <v>0.6193778902879099</v>
       </c>
     </row>
     <row r="184">
@@ -25268,7 +25280,7 @@
         <v>92.0121258530756</v>
       </c>
       <c r="B184" t="n">
-        <v>0.613378341478502</v>
+        <v>0.6133783414785021</v>
       </c>
     </row>
     <row r="185">
@@ -25276,7 +25288,7 @@
         <v>92.9337329950927</v>
       </c>
       <c r="B185" t="n">
-        <v>0.6073198287271747</v>
+        <v>0.6073198287271748</v>
       </c>
     </row>
     <row r="186">
@@ -25284,7 +25296,7 @@
         <v>93.86457109136009</v>
       </c>
       <c r="B186" t="n">
-        <v>0.6012063485759663</v>
+        <v>0.6012063485759664</v>
       </c>
     </row>
     <row r="187">
@@ -25292,7 +25304,7 @@
         <v>94.8047326004888</v>
       </c>
       <c r="B187" t="n">
-        <v>0.595042185078097</v>
+        <v>0.5950421850780969</v>
       </c>
     </row>
     <row r="188">
@@ -25308,7 +25320,7 @@
         <v>96.71340033144673</v>
       </c>
       <c r="B189" t="n">
-        <v>0.5825801894942452</v>
+        <v>0.5825801894942453</v>
       </c>
     </row>
     <row r="190">
@@ -25316,7 +25328,7 @@
         <v>97.6820961380902</v>
       </c>
       <c r="B190" t="n">
-        <v>0.5762920728378665</v>
+        <v>0.5762920728378667</v>
       </c>
     </row>
     <row r="191">
@@ -25324,7 +25336,7 @@
         <v>98.66049454605455</v>
       </c>
       <c r="B191" t="n">
-        <v>0.5699726380274663</v>
+        <v>0.5699726380274664</v>
       </c>
     </row>
     <row r="192">
@@ -25332,7 +25344,7 @@
         <v>99.64869273803822</v>
       </c>
       <c r="B192" t="n">
-        <v>0.5636271199914632</v>
+        <v>0.5636271199914633</v>
       </c>
     </row>
     <row r="193">
@@ -25340,7 +25352,7 @@
         <v>100.6467888701359</v>
       </c>
       <c r="B193" t="n">
-        <v>0.5572608463716293</v>
+        <v>0.5572608463716292</v>
       </c>
     </row>
     <row r="194">
@@ -25348,7 +25360,7 @@
         <v>101.6548820815885</v>
       </c>
       <c r="B194" t="n">
-        <v>0.5508792061991454</v>
+        <v>0.5508792061991455</v>
       </c>
     </row>
     <row r="195">
@@ -25356,7 +25368,7 @@
         <v>102.6730725046301</v>
       </c>
       <c r="B195" t="n">
-        <v>0.5444876195120442</v>
+        <v>0.5444876195120444</v>
       </c>
     </row>
     <row r="196">
@@ -25364,7 +25376,7 @@
         <v>103.7014612744342</v>
       </c>
       <c r="B196" t="n">
-        <v>0.5380915080938837</v>
+        <v>0.5380915080938838</v>
       </c>
     </row>
     <row r="197">
@@ -25372,7 +25384,7 @@
         <v>104.7401505391593</v>
       </c>
       <c r="B197" t="n">
-        <v>0.531696267488981</v>
+        <v>0.5316962674889812</v>
       </c>
     </row>
     <row r="198">
@@ -25388,7 +25400,7 @@
         <v>106.8488442719102</v>
       </c>
       <c r="B199" t="n">
-        <v>0.5189296917462732</v>
+        <v>0.5189296917462733</v>
       </c>
     </row>
     <row r="200">
@@ -25404,7 +25416,7 @@
         <v>108.999991535954</v>
       </c>
       <c r="B201" t="n">
-        <v>0.5062295603510725</v>
+        <v>0.5062295603510724</v>
       </c>
     </row>
     <row r="202">
@@ -25412,7 +25424,7 @@
         <v>110.0917516680887</v>
       </c>
       <c r="B202" t="n">
-        <v>0.4999169149858294</v>
+        <v>0.4999169149858296</v>
       </c>
     </row>
     <row r="203">
@@ -25428,7 +25440,7 @@
         <v>112.308187157011</v>
       </c>
       <c r="B204" t="n">
-        <v>0.4873901247548732</v>
+        <v>0.4873901247548733</v>
       </c>
     </row>
     <row r="205">
@@ -25460,7 +25472,7 @@
         <v>116.8758244714929</v>
       </c>
       <c r="B208" t="n">
-        <v>0.462851097705929</v>
+        <v>0.4628510977059292</v>
       </c>
     </row>
     <row r="209">
@@ -25468,7 +25480,7 @@
         <v>118.0464701180684</v>
       </c>
       <c r="B209" t="n">
-        <v>0.4568461422246426</v>
+        <v>0.4568461422246425</v>
       </c>
     </row>
     <row r="210">
@@ -25476,7 +25488,7 @@
         <v>119.2288411256076</v>
       </c>
       <c r="B210" t="n">
-        <v>0.4508999232968045</v>
+        <v>0.4508999232968044</v>
       </c>
     </row>
     <row r="211">
@@ -25492,7 +25504,7 @@
         <v>121.6292301717424</v>
       </c>
       <c r="B212" t="n">
-        <v>0.4391953424372301</v>
+        <v>0.4391953424372302</v>
       </c>
     </row>
     <row r="213">
@@ -25500,7 +25512,7 @@
         <v>122.8474866370188</v>
       </c>
       <c r="B213" t="n">
-        <v>0.4334421617058021</v>
+        <v>0.4334421617058022</v>
       </c>
     </row>
     <row r="214">
@@ -25508,7 +25520,7 @@
         <v>124.0779453403021</v>
       </c>
       <c r="B214" t="n">
-        <v>0.4277580740402941</v>
+        <v>0.427758074040294</v>
       </c>
     </row>
     <row r="215">
@@ -25516,7 +25528,7 @@
         <v>125.3207285010241</v>
       </c>
       <c r="B215" t="n">
-        <v>0.4221450162275466</v>
+        <v>0.4221450162275467</v>
       </c>
     </row>
     <row r="216">
@@ -25524,7 +25536,7 @@
         <v>126.5759595627839</v>
       </c>
       <c r="B216" t="n">
-        <v>0.4166046619307518</v>
+        <v>0.4166046619307519</v>
       </c>
     </row>
     <row r="217">
@@ -25532,7 +25544,7 @@
         <v>127.8437632056103</v>
       </c>
       <c r="B217" t="n">
-        <v>0.4111384222979433</v>
+        <v>0.4111384222979434</v>
       </c>
     </row>
     <row r="218">
@@ -25540,7 +25552,7 @@
         <v>129.1242653583458</v>
       </c>
       <c r="B218" t="n">
-        <v>0.4057474474556778</v>
+        <v>0.4057474474556779</v>
       </c>
     </row>
     <row r="219">
@@ -25548,7 +25560,7 @@
         <v>130.417593211155</v>
       </c>
       <c r="B219" t="n">
-        <v>0.4004326288427587</v>
+        <v>0.4004326288427588</v>
       </c>
     </row>
     <row r="220">
@@ -25556,7 +25568,7 @@
         <v>131.7238752281579</v>
       </c>
       <c r="B220" t="n">
-        <v>0.3951946023455976</v>
+        <v>0.3951946023455977</v>
       </c>
     </row>
     <row r="221">
@@ -25564,7 +25576,7 @@
         <v>133.0432411601904</v>
       </c>
       <c r="B221" t="n">
-        <v>0.3900337522033527</v>
+        <v>0.3900337522033528</v>
       </c>
     </row>
     <row r="222">
@@ -25580,7 +25592,7 @@
         <v>135.7217502837233</v>
       </c>
       <c r="B223" t="n">
-        <v>0.379943888323491</v>
+        <v>0.3799438883234911</v>
       </c>
     </row>
     <row r="224">
@@ -25604,7 +25616,7 @@
         <v>139.8409625299253</v>
       </c>
       <c r="B226" t="n">
-        <v>0.3653836259950983</v>
+        <v>0.3653836259950982</v>
       </c>
     </row>
     <row r="227">
@@ -25612,7 +25624,7 @@
         <v>141.2416304160244</v>
       </c>
       <c r="B227" t="n">
-        <v>0.3606804866584556</v>
+        <v>0.3606804866584558</v>
       </c>
     </row>
     <row r="228">
@@ -25620,7 +25632,7 @@
         <v>142.6563276000609</v>
       </c>
       <c r="B228" t="n">
-        <v>0.3560506473861167</v>
+        <v>0.3560506473861165</v>
       </c>
     </row>
     <row r="229">
@@ -25644,7 +25656,7 @@
         <v>146.9860071865672</v>
       </c>
       <c r="B231" t="n">
-        <v>0.3425859951533294</v>
+        <v>0.3425859951533295</v>
       </c>
     </row>
     <row r="232">
@@ -25668,7 +25680,7 @@
         <v>151.44709437088</v>
       </c>
       <c r="B234" t="n">
-        <v>0.3297200860148469</v>
+        <v>0.329720086014847</v>
       </c>
     </row>
     <row r="235">
@@ -25684,7 +25696,7 @@
         <v>154.4961212922591</v>
       </c>
       <c r="B236" t="n">
-        <v>0.3214465485690157</v>
+        <v>0.3214465485690158</v>
       </c>
     </row>
     <row r="237">
@@ -25700,7 +25712,7 @@
         <v>157.6065331164382</v>
       </c>
       <c r="B238" t="n">
-        <v>0.3133930040191023</v>
+        <v>0.3133930040191024</v>
       </c>
     </row>
     <row r="239">
@@ -25708,7 +25720,7 @@
         <v>159.185143600676</v>
       </c>
       <c r="B239" t="n">
-        <v>0.3094421321396736</v>
+        <v>0.3094421321396737</v>
       </c>
     </row>
     <row r="240">
@@ -25732,7 +25744,7 @@
         <v>164.0164797097561</v>
       </c>
       <c r="B242" t="n">
-        <v>0.2978601457334238</v>
+        <v>0.2978601457334239</v>
       </c>
     </row>
     <row r="243">
@@ -25740,7 +25752,7 @@
         <v>165.6592931727379</v>
       </c>
       <c r="B243" t="n">
-        <v>0.2940803795509365</v>
+        <v>0.2940803795509364</v>
       </c>
     </row>
     <row r="244">
@@ -25748,7 +25760,7 @@
         <v>167.3185612997812</v>
       </c>
       <c r="B244" t="n">
-        <v>0.2903364008269022</v>
+        <v>0.2903364008269023</v>
       </c>
     </row>
     <row r="245">
@@ -25788,7 +25800,7 @@
         <v>175.8675484545012</v>
       </c>
       <c r="B249" t="n">
-        <v>0.2720583016677415</v>
+        <v>0.2720583016677416</v>
       </c>
     </row>
     <row r="250">
@@ -25796,7 +25808,7 @@
         <v>177.6290639852209</v>
       </c>
       <c r="B250" t="n">
-        <v>0.2684729532296745</v>
+        <v>0.2684729532296746</v>
       </c>
     </row>
     <row r="251">
@@ -25844,7 +25856,7 @@
         <v>188.5749203624483</v>
       </c>
       <c r="B256" t="n">
-        <v>0.2472638342582692</v>
+        <v>0.2472638342582693</v>
       </c>
     </row>
     <row r="257">
@@ -25876,7 +25888,7 @@
         <v>196.2443687315043</v>
       </c>
       <c r="B260" t="n">
-        <v>0.2332892799149434</v>
+        <v>0.2332892799149435</v>
       </c>
     </row>
     <row r="261">
@@ -25956,7 +25968,7 @@
         <v>216.8105342379721</v>
       </c>
       <c r="B270" t="n">
-        <v>0.1985693606837466</v>
+        <v>0.1985693606837467</v>
       </c>
     </row>
     <row r="271">
@@ -25964,7 +25976,7 @@
         <v>218.9821408057555</v>
       </c>
       <c r="B271" t="n">
-        <v>0.1951190901094274</v>
+        <v>0.1951190901094275</v>
       </c>
     </row>
     <row r="272">
@@ -25972,7 +25984,7 @@
         <v>221.1754985080114</v>
       </c>
       <c r="B272" t="n">
-        <v>0.191676119798442</v>
+        <v>0.1916761197984421</v>
       </c>
     </row>
     <row r="273">
@@ -25980,7 +25992,7 @@
         <v>223.3908252073386</v>
       </c>
       <c r="B273" t="n">
-        <v>0.1882417534885085</v>
+        <v>0.1882417534885086</v>
       </c>
     </row>
     <row r="274">
@@ -25996,7 +26008,7 @@
         <v>227.8882679801808</v>
       </c>
       <c r="B275" t="n">
-        <v>0.1814046250325867</v>
+        <v>0.1814046250325866</v>
       </c>
     </row>
     <row r="276">
@@ -26012,7 +26024,7 @@
         <v>232.4762560629131</v>
       </c>
       <c r="B277" t="n">
-        <v>0.1746202906389593</v>
+        <v>0.1746202906389594</v>
       </c>
     </row>
     <row r="278">
@@ -26020,7 +26032,7 @@
         <v>234.804772831226</v>
       </c>
       <c r="B278" t="n">
-        <v>0.1712522326487497</v>
+        <v>0.1712522326487498</v>
       </c>
     </row>
     <row r="279">
@@ -26044,7 +26056,7 @@
         <v>241.9311965156471</v>
       </c>
       <c r="B281" t="n">
-        <v>0.1612667015765813</v>
+        <v>0.1612667015765812</v>
       </c>
     </row>
     <row r="282">
@@ -26068,7 +26080,7 @@
         <v>249.273910158392</v>
       </c>
       <c r="B284" t="n">
-        <v>0.1514997247126441</v>
+        <v>0.1514997247126442</v>
       </c>
     </row>
     <row r="285">
@@ -26076,7 +26088,7 @@
         <v>251.7706747292632</v>
       </c>
       <c r="B285" t="n">
-        <v>0.1483017726338731</v>
+        <v>0.1483017726338732</v>
       </c>
     </row>
     <row r="286">
@@ -26172,7 +26184,7 @@
         <v>283.7559357900884</v>
       </c>
       <c r="B297" t="n">
-        <v>0.112930125306664</v>
+        <v>0.1129301253066641</v>
       </c>
     </row>
     <row r="298">
@@ -26212,7 +26224,7 @@
         <v>298.254182914021</v>
       </c>
       <c r="B302" t="n">
-        <v>0.100190086571232</v>
+        <v>0.1001900865712321</v>
       </c>
     </row>
     <row r="303">
@@ -26220,7 +26232,7 @@
         <v>301.2415411840486</v>
       </c>
       <c r="B303" t="n">
-        <v>0.09779972704876201</v>
+        <v>0.09779972704876203</v>
       </c>
     </row>
     <row r="304">
@@ -26228,7 +26240,7 @@
         <v>304.2588212789656</v>
       </c>
       <c r="B304" t="n">
-        <v>0.09546273280796229</v>
+        <v>0.0954627328079623</v>
       </c>
     </row>
     <row r="305">
@@ -26236,7 +26248,7 @@
         <v>307.3063229002207</v>
       </c>
       <c r="B305" t="n">
-        <v>0.09317919995087776</v>
+        <v>0.09317919995087777</v>
       </c>
     </row>
     <row r="306">
@@ -26244,7 +26256,7 @@
         <v>310.3843487511191</v>
       </c>
       <c r="B306" t="n">
-        <v>0.09094909958975267</v>
+        <v>0.09094909958975264</v>
       </c>
     </row>
     <row r="307">
@@ -26260,7 +26272,7 @@
         <v>316.633199145035</v>
       </c>
       <c r="B308" t="n">
-        <v>0.08664846948894994</v>
+        <v>0.08664846948894996</v>
       </c>
     </row>
     <row r="309">
@@ -26276,7 +26288,7 @@
         <v>323.0078552743323</v>
       </c>
       <c r="B310" t="n">
-        <v>0.08255821024285169</v>
+        <v>0.08255821024285166</v>
       </c>
     </row>
     <row r="311">
@@ -26284,7 +26296,7 @@
         <v>326.2431500095479</v>
       </c>
       <c r="B311" t="n">
-        <v>0.08059065240034251</v>
+        <v>0.08059065240034254</v>
       </c>
     </row>
     <row r="312">
@@ -26292,7 +26304,7 @@
         <v>329.5108499381753</v>
       </c>
       <c r="B312" t="n">
-        <v>0.07867389528168459</v>
+        <v>0.0786738952816846</v>
       </c>
     </row>
     <row r="313">
@@ -26308,7 +26320,7 @@
         <v>336.1447669276134</v>
       </c>
       <c r="B314" t="n">
-        <v>0.0749894613804049</v>
+        <v>0.07498946138040491</v>
       </c>
     </row>
     <row r="315">
@@ -26316,7 +26328,7 @@
         <v>339.5116429244453</v>
       </c>
       <c r="B315" t="n">
-        <v>0.07321990371840002</v>
+        <v>0.07321990371840005</v>
       </c>
     </row>
     <row r="316">
@@ -26332,7 +26344,7 @@
         <v>346.346902086719</v>
       </c>
       <c r="B317" t="n">
-        <v>0.06982081681899048</v>
+        <v>0.06982081681899049</v>
       </c>
     </row>
     <row r="318">
@@ -26340,7 +26352,7 @@
         <v>349.8159641871673</v>
       </c>
       <c r="B318" t="n">
-        <v>0.06818896693567562</v>
+        <v>0.0681889669356756</v>
       </c>
     </row>
     <row r="319">
@@ -26348,7 +26360,7 @@
         <v>353.319772929738</v>
       </c>
       <c r="B319" t="n">
-        <v>0.06660060314056128</v>
+        <v>0.06660060314056124</v>
       </c>
     </row>
     <row r="320">
@@ -26372,7 +26384,7 @@
         <v>364.0431767499432</v>
       </c>
       <c r="B322" t="n">
-        <v>0.06208332113312456</v>
+        <v>0.06208332113312457</v>
       </c>
     </row>
     <row r="323">
@@ -26388,7 +26400,7 @@
         <v>371.3723199802301</v>
       </c>
       <c r="B324" t="n">
-        <v>0.05926466849580083</v>
+        <v>0.05926466849580081</v>
       </c>
     </row>
     <row r="325">
@@ -26396,7 +26408,7 @@
         <v>375.0920403895569</v>
       </c>
       <c r="B325" t="n">
-        <v>0.05790901867885429</v>
+        <v>0.05790901867885431</v>
       </c>
     </row>
     <row r="326">
@@ -26404,7 +26416,7 @@
         <v>378.8490180719203</v>
       </c>
       <c r="B326" t="n">
-        <v>0.05658728180675916</v>
+        <v>0.05658728180675917</v>
       </c>
     </row>
     <row r="327">
@@ -26412,7 +26424,7 @@
         <v>382.6436262017089</v>
       </c>
       <c r="B327" t="n">
-        <v>0.05529806314402084</v>
+        <v>0.05529806314402085</v>
       </c>
     </row>
     <row r="328">
@@ -26420,7 +26432,7 @@
         <v>386.4762416910843</v>
       </c>
       <c r="B328" t="n">
-        <v>0.05403998360222882</v>
+        <v>0.05403998360222884</v>
       </c>
     </row>
     <row r="329">
@@ -26428,7 +26440,7 @@
         <v>390.3472452274132</v>
       </c>
       <c r="B329" t="n">
-        <v>0.052811686521548</v>
+        <v>0.05281168652154802</v>
       </c>
     </row>
     <row r="330">
@@ -26436,7 +26448,7 @@
         <v>394.2570213110868</v>
       </c>
       <c r="B330" t="n">
-        <v>0.05161184406989549</v>
+        <v>0.0516118440698955</v>
       </c>
     </row>
     <row r="331">
@@ -26444,7 +26456,7 @@
         <v>398.2059582937063</v>
       </c>
       <c r="B331" t="n">
-        <v>0.05043916321945573</v>
+        <v>0.05043916321945574</v>
       </c>
     </row>
     <row r="332">
@@ -26452,7 +26464,7 @@
         <v>402.1944484166634</v>
       </c>
       <c r="B332" t="n">
-        <v>0.04929239126433066</v>
+        <v>0.04929239126433067</v>
       </c>
     </row>
     <row r="333">
@@ -26460,7 +26472,7 @@
         <v>406.2228878500953</v>
       </c>
       <c r="B333" t="n">
-        <v>0.04817032084763447</v>
+        <v>0.04817032084763448</v>
       </c>
     </row>
     <row r="334">
@@ -26468,7 +26480,7 @@
         <v>410.2916767322396</v>
       </c>
       <c r="B334" t="n">
-        <v>0.0470717944711033</v>
+        <v>0.04707179447110332</v>
       </c>
     </row>
     <row r="335">
@@ -26492,7 +26504,7 @@
         <v>422.7442018122436</v>
       </c>
       <c r="B337" t="n">
-        <v>0.04390673194950059</v>
+        <v>0.0439067319495006</v>
       </c>
     </row>
     <row r="338">
@@ -26508,7 +26520,7 @@
         <v>431.2551505203514</v>
       </c>
       <c r="B339" t="n">
-        <v>0.0418957540251039</v>
+        <v>0.04189575402510391</v>
       </c>
     </row>
     <row r="340">
@@ -26524,7 +26536,7 @@
         <v>439.9374469313995</v>
       </c>
       <c r="B341" t="n">
-        <v>0.03995615783849189</v>
+        <v>0.03995615783849187</v>
       </c>
     </row>
     <row r="342">
@@ -26548,7 +26560,7 @@
         <v>453.2897336148099</v>
       </c>
       <c r="B344" t="n">
-        <v>0.03716870732068531</v>
+        <v>0.03716870732068532</v>
       </c>
     </row>
     <row r="345">
@@ -26556,7 +26568,7 @@
         <v>457.8299510266926</v>
       </c>
       <c r="B345" t="n">
-        <v>0.03626987479979618</v>
+        <v>0.03626987479979617</v>
       </c>
     </row>
     <row r="346">
@@ -26572,7 +26584,7 @@
         <v>467.0472678190211</v>
       </c>
       <c r="B347" t="n">
-        <v>0.03451513183473646</v>
+        <v>0.03451513183473644</v>
       </c>
     </row>
     <row r="348">
@@ -26596,7 +26608,7 @@
         <v>481.2223489768562</v>
       </c>
       <c r="B350" t="n">
-        <v>0.03198587034190424</v>
+        <v>0.03198587034190425</v>
       </c>
     </row>
     <row r="351">
@@ -26612,7 +26624,7 @@
         <v>490.9106160465869</v>
       </c>
       <c r="B352" t="n">
-        <v>0.03036598479569731</v>
+        <v>0.03036598479569732</v>
       </c>
     </row>
     <row r="353">
@@ -26620,7 +26632,7 @@
         <v>495.8276498141029</v>
       </c>
       <c r="B353" t="n">
-        <v>0.02957560841457882</v>
+        <v>0.02957560841457883</v>
       </c>
     </row>
     <row r="354">
@@ -26628,7 +26640,7 @@
         <v>500.7939333233867</v>
       </c>
       <c r="B354" t="n">
-        <v>0.02879822124105335</v>
+        <v>0.02879822124105336</v>
       </c>
     </row>
     <row r="355">
@@ -26644,7 +26656,7 @@
         <v>510.8762276791109</v>
       </c>
       <c r="B356" t="n">
-        <v>0.02728242996791174</v>
+        <v>0.02728242996791175</v>
       </c>
     </row>
     <row r="357">
@@ -26692,7 +26704,7 @@
         <v>542.3574373936458</v>
       </c>
       <c r="B362" t="n">
-        <v>0.02305085336726235</v>
+        <v>0.02305085336726236</v>
       </c>
     </row>
     <row r="363">
@@ -26700,7 +26712,7 @@
         <v>547.7897701779814</v>
       </c>
       <c r="B363" t="n">
-        <v>0.02239252462213946</v>
+        <v>0.02239252462213945</v>
       </c>
     </row>
     <row r="364">
@@ -26708,7 +26720,7 @@
         <v>553.276514015702</v>
       </c>
       <c r="B364" t="n">
-        <v>0.0217478537916932</v>
+        <v>0.02174785379169321</v>
       </c>
     </row>
     <row r="365">
@@ -26748,7 +26760,7 @@
         <v>581.5456658335572</v>
       </c>
       <c r="B369" t="n">
-        <v>0.01873199268834814</v>
+        <v>0.01873199268834815</v>
       </c>
     </row>
     <row r="370">
@@ -26804,7 +26816,7 @@
         <v>623.5654535780452</v>
       </c>
       <c r="B376" t="n">
-        <v>0.0150953736018849</v>
+        <v>0.01509537360188491</v>
       </c>
     </row>
     <row r="377">
@@ -26828,7 +26840,7 @@
         <v>642.4909275519475</v>
       </c>
       <c r="B379" t="n">
-        <v>0.01374245140721105</v>
+        <v>0.01374245140721104</v>
       </c>
     </row>
     <row r="380">
@@ -26836,7 +26848,7 @@
         <v>648.9262122714705</v>
       </c>
       <c r="B380" t="n">
-        <v>0.01331798489020889</v>
+        <v>0.0133179848902089</v>
       </c>
     </row>
     <row r="381">
@@ -26868,7 +26880,7 @@
         <v>675.3184073246478</v>
       </c>
       <c r="B384" t="n">
-        <v>0.0117475557285111</v>
+        <v>0.01174755572851109</v>
       </c>
     </row>
     <row r="385">
@@ -26916,7 +26928,7 @@
         <v>716.9328713635316</v>
       </c>
       <c r="B390" t="n">
-        <v>0.009747813097161179</v>
+        <v>0.009747813097161181</v>
       </c>
     </row>
     <row r="391">
@@ -26924,7 +26936,7 @@
         <v>724.11377766767</v>
       </c>
       <c r="B391" t="n">
-        <v>0.009452564890521768</v>
+        <v>0.009452564890521769</v>
       </c>
     </row>
     <row r="392">
@@ -26940,7 +26952,7 @@
         <v>738.6920857654368</v>
       </c>
       <c r="B393" t="n">
-        <v>0.008892033986567797</v>
+        <v>0.008892033986567799</v>
       </c>
     </row>
     <row r="394">
@@ -26956,7 +26968,7 @@
         <v>753.5638934119596</v>
       </c>
       <c r="B395" t="n">
-        <v>0.008369437713890603</v>
+        <v>0.008369437713890605</v>
       </c>
     </row>
     <row r="396">
@@ -26972,7 +26984,7 @@
         <v>768.7351095223567</v>
       </c>
       <c r="B397" t="n">
-        <v>0.007882343033713235</v>
+        <v>0.007882343033713237</v>
       </c>
     </row>
     <row r="398">
@@ -26988,7 +27000,7 @@
         <v>784.2117619736939</v>
       </c>
       <c r="B399" t="n">
-        <v>0.007428331203824577</v>
+        <v>0.007428331203824578</v>
       </c>
     </row>
     <row r="400">
@@ -27004,7 +27016,7 @@
         <v>800.0000000000003</v>
       </c>
       <c r="B401" t="n">
-        <v>0.007005022227457485</v>
+        <v>0.007005022227457487</v>
       </c>
     </row>
   </sheetData>

</xml_diff>